<commit_message>
Fix occupancy precision (store ratios at 4 dp)
Occupancy showed rounded values (e.g. 95.00% instead of 94.83%) for two
reasons: the seeded ratios were rounded to 2 dp, and RevenueSummary's value
columns were Decimal(18,2) so they could not hold more precision anyway.

- schema: RevenueSummary actual/budget/lastYear → Decimal(18,4)
- seed-data: real MTD occupancy ratios to 4 dp (BKDS 0.8407/0.9019,
  BKDU 0.9483/0.9317, BKV 0.8289/0.9022), read unrounded from the workbooks
- migration widen_revenue_summary_precision; regenerated seed.sql + sample
- Money is unaffected (2 dp values just carry .0000)

Typecheck, 32 tests, and build all pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CnH3YBKxFBiwcDeXQMi11x
</commit_message>
<xml_diff>
--- a/samples/BK_SalesData_BKDS_2026-06.xlsx
+++ b/samples/BK_SalesData_BKDS_2026-06.xlsx
@@ -439,10 +439,10 @@
         <v>OCCUPANCY</v>
       </c>
       <c r="B2">
-        <v>0.84</v>
+        <v>0.8407</v>
       </c>
       <c r="C2">
-        <v>0.9</v>
+        <v>0.9019</v>
       </c>
       <c r="D2" t="str">
         <v/>

</xml_diff>